<commit_message>
Add GLDComplianceAdapterServices analysis and updated map field mappings
- WebMethods/Analysis/GLDComplianceAdapterServices_Analysis.md: component-level analysis
  of all 7 JDBC adapter services (logCheckRequest, logCheckRequestXML, logCheckReply,
  logCheckReplyError, selectCustomerAndRequest, updateCIURefNbr, purgeData) with full
  field tables, SQL, and connection details
- WebMethods/MD/PackageAnalysis.md: comprehensive Boomi migration reference (~300 lines)
  with 9 component definitions, DDPs, Map field mapping table, DB schema, and gap analysis
- WebMethods/Analysis/map_field_mappings.xlsx: updated with actual pipeline fields from
  GLDComplianceAdapterServices (logCheckRequest 26-row, selectCustomerAndRequest 25-row,
  logCheckReplyError 4-row sheets + Instructions tab)
- scripts/gen_gld_cas_map_excel.py: generator script for the above Excel

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WebMethods/Analysis/map_field_mappings.xlsx
+++ b/WebMethods/Analysis/map_field_mappings.xlsx
@@ -7,8 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Map Field Mappings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="logCheckRequest" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="selectCustomerAndRequest" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="logCheckReplyError" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Instructions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -447,14 +449,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="58" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,7 +489,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>COMPLIANCE_RECORDS/RECORD_ID</t>
+          <t>request/CustomerNbr</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -497,24 +499,20 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>complianceOutput/recordId</t>
+          <t>CUSTOMERNBR</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Primary key -- no transformation needed.</t>
-        </is>
-      </c>
+          <t>VARCHAR2(18)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>COMPLIANCE_RECORDS/ENTITY_ID</t>
+          <t>request/CustomerType</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -524,51 +522,43 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>complianceOutput/entityId</t>
+          <t>CUSTOMERTYPE</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Entity identifier.</t>
-        </is>
-      </c>
+          <t>VARCHAR2(3)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>COMPLIANCE_RECORDS/COMPLIANCE_STATUS</t>
+          <t>request/PartyType</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Lookup translate: PASS -&gt; Approved; FAIL -&gt; Rejected; PENDING -&gt; Under_Review</t>
+          <t>Direct copy</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>complianceOutput/status</t>
+          <t>PARTYTYPE</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Status code translation. Implement as a Cross-Reference Table in Boomi.</t>
-        </is>
-      </c>
+          <t>VARCHAR2(20)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>COMPLIANCE_RECORDS/REVIEWED_BY</t>
+          <t>request/Businessname</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -578,59 +568,543 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>complianceOutput/reviewedBy</t>
+          <t>BUSINESSNAME</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>Reviewer name.</t>
-        </is>
-      </c>
+          <t>VARCHAR2(40)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>COMPLIANCE_RECORDS/REVIEW_DATE</t>
+          <t>request/ApplicationNbr</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Date format: yyyy-MM-dd HH:mm:ss -&gt; yyyy-MM-ddTHH:mm:ssZ (ISO-8601)</t>
+          <t>Direct copy</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>complianceOutput/reviewDate</t>
+          <t>APPLICATIONNBR</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>DATETIME</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Use Boomi Map date/time function: CurrentDateTimeToFormat with target mask.</t>
-        </is>
-      </c>
+          <t>VARCHAR2(18)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr"/>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>request/Channel</t>
+        </is>
+      </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>--- Template row: add actual MAP step pipeline fields below ---</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>No MAP steps were found in GLDComplianceAdapterEnv (only a JDBC connection node). Populate when flow services with MAP steps are available.</t>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>CHANNEL</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>VARCHAR2(10)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>request/LOB</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>LOB</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR2(10)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>request/ProductCode</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>PRODUCTCODE</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>VARCHAR2(10)</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>request/SubProductCode</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>SUBPRODUCTCODE</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR2(10)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>request/PostBack</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>POSTBACK</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>VARCHAR2(200)</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>request/ComplianceReplyEmail</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>COMPLIANCEREPLYEMAIL</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR2(75)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>request/FirstName</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>FIRSTNAME</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>VARCHAR2(20)</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>request/MiddleName</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>MIDDLENAME</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR2(20)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>request/LastName</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>LASTNAME</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>VARCHAR2(20)</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>request/AddressLine1</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>ADDRESSLINE1</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR2(40)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>request/AddressLine2</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>ADDRESSLINE2</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>VARCHAR2(40)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>request/AddressLine3</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>ADDRESSLINE3</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR2(40)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>request/AddressLine4</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>ADDRESSLINE4</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>VARCHAR2(40)</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>request/City</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>CITY</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR2(20)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>request/State</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>STATE</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>VARCHAR2(2)</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>2-char state code</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>request/Zip</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>ZIP</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR2(10)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>request/CountryCode</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>COUNTRYCODE</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>VARCHAR2(3)</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>3-char ISO code</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>request/SSNTIN</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy (PII — do not log)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>SSNTIN</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR2(9)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>SSN or TIN. Set enableUserLog=false on process.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>request/DOB</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Date format: input yyyy-MM-dd → Oracle DATE</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>DOB</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Use Boomi Map CurrentDateTimeToFormat function</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>request/RequestorSystemRequestID</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Convert String to Long</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>REQUESTORSYSTEMREQUESTID</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>BIGINT</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Cast using Boomi Map Number function</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>(OUT) Oracle auto-generated</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Returned by SP</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>accCheckRequestID</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Long/BIGINT</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Store as DPP_ACC_CHECK_REQUEST_ID for later use</t>
         </is>
       </c>
     </row>
@@ -645,7 +1119,794 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source (Pipeline In)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Transformation Logic</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Target (Pipeline Out)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>DPP_CIU_REF_NBR</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy → SQL WHERE param</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>WHERE t2.CIUREFNBR = ?</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR2(20)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Set before calling this operation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>results[]/ACCCUSTOMERID</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>DPP_ACC_CUSTOMER_ID</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>BigDecimal</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>results[]/CUSTOMERNBR</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>DPP_CUSTOMER_NBR</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>results[]/CUSTOMERTYPE</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>DPP_CUSTOMER_TYPE</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>results[]/BUSINESSNAME</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>DPP_BUSINESS_NAME</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>results[]/FIRSTNAME</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>DPP_FIRST_NAME</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>results[]/MIDDLENAME</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>DPP_MIDDLE_NAME</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>results[]/LASTNAME</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>DPP_LAST_NAME</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>results[]/ADDRESSLINE1</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>DPP_ADDRESS_LINE1</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>results[]/ADDRESSLINE2</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>DPP_ADDRESS_LINE2</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>results[]/CITY</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>DPP_CITY</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>results[]/STATE</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>DPP_STATE</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>results[]/ZIP</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>DPP_ZIP</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>results[]/SSNTIN</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy (PII)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>DPP_SSNTIN</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Handle as sensitive data</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>results[]/DOB</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp → String yyyy-MM-dd</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>DPP_DOB</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>results[]/PARTYTYPE</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>DPP_PARTY_TYPE</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>results[]/ACCCHECKREQUESTID</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>DPP_ACC_CHECK_REQUEST_ID</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BigDecimal</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>results[]/APPLICATIONNBR</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>DPP_APPLICATION_NBR</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>results[]/CHANNEL</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>DPP_CHANNEL</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>results[]/LOB</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>DPP_LOB</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>results[]/PRODUCTCODE</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>DPP_PRODUCT_CODE</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>results[]/SUBPRODUCTCODE</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>DPP_SUB_PRODUCT_CODE</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>results[]/COMPLIANCEREPLYEMAIL</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>DPP_COMPLIANCE_REPLY_EMAIL</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>results[]/CIUREFNBR</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>DPP_CIU_REF_NBR</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Confirm matches input</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>results[]/REQUESTTIMESTAMP</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp → ISO-8601 String</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>DPP_REQUEST_TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Use CurrentDateTimeToFormat</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Source (Pipeline In)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Transformation Logic</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Target (Pipeline Out)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>$error/errorMessage</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ERRORDESC</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>webMethods $error pipeline variable</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>$error/errorCode</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>ERRORCODE</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>$error/errorType</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ERRORTYPE</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>DPP_CIU_REF_NBR</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Direct copy</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>CIUREFNBR</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Must be set before entering error path</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -664,83 +1925,83 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>This file documents MAP shape field mappings for the webMethods -&gt; Boomi GLD Compliance migration.</t>
+          <t>Package: GLDComplianceAdapterServices (webMethods IS 6.5, Oracle JDBC adapter)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Generated from node.ndf analysis of all 7 adapter services.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Column descriptions:</t>
-        </is>
-      </c>
+      <c r="A5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Source (Pipeline In)     — Field path from the webMethods pipeline input document.</t>
+          <t>Sheets:</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Transformation Logic     — Script, formula, lookup, or "Direct copy" used to derive output.</t>
+          <t xml:space="preserve">  logCheckRequest           — Maps input request document fields to ACCLOGCHECKREQUEST SP parameters</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Target (Pipeline Out)    — Field path in the Boomi output document / JSON profile.</t>
+          <t xml:space="preserve">  selectCustomerAndRequest  — Maps CIURefNbr input and output row fields from the JOIN SELECT query</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Data Type                — webMethods IS data type (STRING, INTEGER, DATETIME, OBJECT, etc.)</t>
+          <t xml:space="preserve">  logCheckReplyError        — Maps error pipeline to ACCLOGCHECKREPLYERROR SP parameters</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Notes                    — Edge cases, TODO items, or Boomi Map function references.</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Sheets not included (direct-copy or void SPs):</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Source package: GLDComplianceAdapterEnv (webMethods IS 6.5, keybank.com, 2008-03-27)</t>
+          <t xml:space="preserve">  logCheckReply      — IN: CIURefNbr (String), CheckType (String), Result (Boolean→VARCHAR2)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>No MAP steps were found in the analyzed package (only a JDBC adapter connection node).</t>
+          <t xml:space="preserve">  logCheckRequestXML — IN: ApplicationID (Long), Request (CLOB), RequestIdentifier1/2/3 (String)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>The rows in the Map Field Mappings sheet are representative placeholders.</t>
+          <t xml:space="preserve">  updateCIURefNbr    — IN: accCheckRequestID (Long), CIURefNbr (String)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Populate them when flow services containing MAP steps are provided.</t>
+          <t xml:space="preserve">  purgeData          — No inputs or outputs</t>
         </is>
       </c>
     </row>
@@ -750,7 +2011,42 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Boomi Map documentation: https://help.boomi.com/docs/atomsphere/integration/process-building/r-atm-map_shape_0abe324f-c3b6-437c-aeac-b6c1c7d5d0a4/</t>
+          <t>Column descriptions:</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Source (Pipeline In)    — webMethods pipeline variable or DB result field</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Transformation Logic    — "Direct copy", date format, type cast, or formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Target (Pipeline Out)   — Boomi DDP name or DB column/SP parameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Data Type               — Oracle or Java data type</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Notes                   — PII flags, format requirements, Boomi Map function hints</t>
         </is>
       </c>
     </row>

</xml_diff>